<commit_message>
docs: 新增Google Workspace MCP配置、Cloud凭证创建指南
- 环境配置文档新增 Google Workspace MCP（Sheets/Docs/Drive/Gmail）安装说明
- 新增 Google Cloud OAuth 凭证创建中文引导文档（含逐步截图式操作）
- 竞品清单更新

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-AI营销/04-选品库/C端/01-疗愈水晶手链/01-竞品分析/1A-竞品清单.xlsx
+++ b/01-AI营销/04-选品库/C端/01-疗愈水晶手链/01-竞品分析/1A-竞品清单.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -526,12 +526,13 @@
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="35" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>疗愈水晶项目 - 竞争对手总览（30家）</t>
+          <t>疗愈水晶手链项目 - 竞品清单（共41家）</t>
         </is>
       </c>
     </row>
@@ -596,6 +597,11 @@
           <t>深度拆解文档</t>
         </is>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>参考重点</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -658,6 +664,11 @@
           <t>P0-1-Loner-Wolf深度拆解.md</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>参考：4层渐进内容框架 × 42个免费测试 × 3层变现 × 反广告品牌定位</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -720,6 +731,11 @@
           <t>P0-2-Daily-Horoscope深度拆解.md</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>参考：内容矩阵乘法(192页) × 5层Freemium漏斗 × 9个互动工具 × 20+数字产品</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -782,6 +798,11 @@
           <t>P0-3-Soul-Path深度拆解.md</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>参考：事件驱动内容模式 × 泛灵性矩阵 × 买量ROI验证 × 极简技术方案</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -844,6 +865,11 @@
           <t>P0-4-Forever-Conscious深度拆解.md</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>参考：月相内容节奏 × 仪式模板 × $5.99月度解读 × 月历产品 × 5层变现</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -906,6 +932,11 @@
           <t>P0-5-Moon-Omens深度拆解.md</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>参考：3站架构 × MemberPress会员 × 9个电子书 × 免费会员每日内容 × 3个免费诱饵</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -968,6 +999,11 @@
           <t>P0-6-Tarot-com深度拆解.md</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>参考：6类每日内容(28页/天) × Freemium抽牌 × Karma Coins虚拟货币 × 姐妹站网络</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1030,6 +1066,11 @@
           <t>P1-1-Energy-Muse深度拆解.md</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>参考：Shop by Intention 8意图分类 × Crystal Test × 名人背书 × KOL矩阵</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1092,6 +1133,11 @@
           <t>P1-2-Healing-Crystals深度拆解.md</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>参考：7维标签系统 × Metaphysical Guide百科 × 批发模式 × 联盟营销 × 4搜索框</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1154,6 +1200,11 @@
           <t>P1-3-Ceremonia深度拆解.md</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>参考：(域名已停放，不再运营)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1216,6 +1267,11 @@
           <t>P1-4-Mindbodygreen深度拆解.md</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>参考：30+MD/PhD Faculty × 113k学员课程 × 1M+订阅者Newsletter × 5频道内容</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1278,6 +1334,11 @@
           <t>P1-5-Selfgazer深度拆解.md</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>参考：心理学+灵性融合 × AI占卜工具 × 图表可视化 × 竞品对比SEO</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1340,6 +1401,11 @@
           <t>P1-6-Mindvalley深度拆解.md</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>参考：Quest微学习模式 × 200+教师网络 × $399/年会员 × 品牌生态系统</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1402,6 +1468,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>参考：天使号码文章SEO × 宝石手链132款 × 按产品形态+水晶双维度分类</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1464,6 +1535,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>参考：石头列表A-Z百科 × 诗意命名 × Crystal Energy产品线 × 课程 × 电台</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1526,6 +1602,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>参考：水晶摆件/礼品收藏品参考 (网站停更)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1588,6 +1669,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>参考：500+水晶数据库 × 7维度搜索 × Crystal Identifier App × 订阅盒 × Premium会员</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1650,6 +1736,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>参考：60+功效文章 × 100水晶A-Z × 10种形状指南 × 伦理采购 × Mystery Box</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1712,6 +1803,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>参考：(已移除 - 珠宝材料批发商)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1774,6 +1870,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>参考：Crystal Quiz × Healing Lamps × 3步漏斗 × 对比营销 × 每单种树 × 多语言</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1836,6 +1937,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>参考：道德采购核心差异化 × 245+水晶完整指南 × NYT引用 × 创始人个人品牌</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1898,6 +2004,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>参考：7大品类全覆盖 × 中国生肖套装 × Adopt a Stone慈善 × 9层变现 × 蜡烛交叉</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1960,6 +2071,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>参考：106种宝石含义 × 30+功效分类 × 12色分类 × 联盟变现 × Printable Cards</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2022,6 +2138,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>参考：100+宝石A-Z × 15意图 × 17色 × 7脉轮 × Moldavite专家 × VIP Club</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -2084,6 +2205,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>参考：MBTI性格测试 × 关系教练 × 5708对成功匹配 × 11M社区</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -2146,6 +2272,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>参考：灵性+健康双品牌 × 24种语言 × 6个计算器工具 × 水晶内容</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -2208,6 +2339,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>参考：Angel Numbers内容工厂(3200+篇) × Eugene个人品牌</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -2270,6 +2406,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>参考：78张塔罗牌全覆盖 × 灵性生活方式 × 含水晶内容</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -2332,6 +2473,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>参考：轻量级博客型 × Angel Numbers+星座 × 后期直接抄</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
@@ -2392,6 +2538,748 @@
       <c r="L31" s="10" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>参考：WordPress+Elementor × 星座+塔罗+号码 × 5个交互工具 × Birthstones × Shop</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>P3-B</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>P3-B-1</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Biddy Tarot</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>biddytarot.com</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>~70</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>~3M</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>内容媒体+课程+认证</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>78牌×多维度内容矩阵(468+页) × 3路径漏斗 × Brigit个人品牌 × 认证体系</t>
+        </is>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>P3-B-1-Biddy-Tarot深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>参考：78牌×多维度内容矩阵(468+页) × 3路径用户漏斗 × Brigit个人品牌 × 认证体系 × Raptive广告</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>P3-B</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>P3-B-2</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Labyrinthos</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>labyrinthos.co</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>~500K</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>App+牌面+工作簿</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>免费App驱动 × 6副牌产品线 × 数字工作簿PDF × App到实体牌变现</t>
+        </is>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>P3-B-2-Labyrinthos深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>参考：免费App驱动 × 6副牌产品线 × 数字工作簿PDF × App到实体牌变现 × Shopify</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>P3-B</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>P3-B-3</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>The Tarot Lady</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>thetarotlady.com</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>~55</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>~300K</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>个人品牌+书籍+播客</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>Theresa 30年个人品牌 × 10本书 × 3个播客 × Patreon × 10+媒体引用</t>
+        </is>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>P3-B-3-The-Tarot-Lady深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>参考：30年个人品牌 × 10本书 × 3个播客 × Patreon会员 × 免费eBook诱饵 × NBC等10+媒体引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>P3-C</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>P3-C-1</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Astrostyle</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>astrostyle.com</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>~75</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>~5M</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>内容媒体+书籍+广告</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>ELLE官方占星师 × I*AM性格测试(3原型) × 每日/周/月运势矩阵 × 畅销书</t>
+        </is>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L35" s="12" t="inlineStr">
+        <is>
+          <t>P3-C-1-Astrostyle深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>参考：ELLE官方占星师背书 × I*AM性格测试(3原型) × 12星座×日/周/月矩阵 × 畅销书 × AdThrive广告</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>P3-C</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>P3-C-2</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Cafe Astrology</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>cafeastrology.nyc</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>~70</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>~3M</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>免费工具+付费报告</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>免费星盘生成器 × 12×12配对矩阵(144页) × 传统占星学教育 × 付费报告</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>P3-C-2-Cafe-Astrology深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>参考：免费星盘生成器(高搜索意图) × 12×12配对矩阵(144页) × 传统占星学教育 × 付费报告</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>P3-D</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>P3-D-1</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Dream Moods</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>dreammoods.com</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>~70</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>~2M</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>静态HTML</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>广告+内容</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>6000+梦典符号 × 26主题分类 × 论坛 × 5大梦论理论家</t>
+        </is>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>P3-D-1-Dream-Moods深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>参考：6000+梦典A-Z × 26主题分类 × 论坛3版块 × 长青静态HTML(停更仍~2M流量)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>P3-D</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>P3-D-2</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Dream Bible</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>dreambible.com</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>~500K</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>静态HTML</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>广告+内容</t>
+        </is>
+      </c>
+      <c r="J38" s="12" t="inlineStr">
+        <is>
+          <t>6406在线符号(2025活跃更新) × ChatGPT辅助研究 × Gillian Holloway Ph.D启发</t>
+        </is>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr">
+        <is>
+          <t>P3-D-2-Dream-Bible深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>参考：6406在线符号(2025活跃更新) × ChatGPT辅助内容生产 × 学术权威背书 × 多国注册商标</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>P3-D</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>P3-D-3</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Dream Dictionary</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>dreamdictionary.org</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>~45</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>~300K</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>工具+广告</t>
+        </is>
+      </c>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>免费在线梦分析工具 × Jung/Freud理论基础 × 原型符号内容</t>
+        </is>
+      </c>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>P3-D-3-Dream-Dictionary深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>参考：免费在线梦分析工具 × Jung/Freud理论基础 × 原型符号(Ouroboros/Phoenix等) × WordPress</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>P3-E</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>P3-E-1</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Tiny Buddha</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>tinybuddha.com</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>~80</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>~10M</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>内容媒体+Shop</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>"Simple wisdom"简约定位 × 8大博客分类 × 论坛3版块 × 3款日记本 × PWYC定价</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L40" s="12" t="inlineStr">
+        <is>
+          <t>P3-E-1-Tiny-Buddha深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>参考："Simple wisdom"简约定位 × 8大博客分类 × 论坛3版块 × 3款日记本Shop × PWYC灵活定价 × ~10M流量</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>P3-E</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>P3-E-2</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Ask-Angels</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>ask-angels.com</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>~55</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>~500K</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>内容+课程+解读</t>
+        </is>
+      </c>
+      <c r="J41" s="12" t="inlineStr">
+        <is>
+          <t>Melanie个人品牌 × 免费天使牌阅读 × 天使传讯系统 × #1播客 × 6层变现</t>
+        </is>
+      </c>
+      <c r="K41" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L41" s="12" t="inlineStr">
+        <is>
+          <t>P3-E-2-Ask-Angels深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>参考：Melanie个人品牌 × 免费天使牌阅读工具 × 天使传讯系统 × #1播客 × 6层变现 × 11:11内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>P3-E</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>P3-E-3</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>The Hoodwitch</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>thehoodwitch.com</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>~300K</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>Squarespace</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>内容+美学品牌</t>
+        </is>
+      </c>
+      <c r="J42" s="12" t="inlineStr">
+        <is>
+          <t>现代巫术美学 × Bri Luna创始人 × Witch Tips每周运势 × 月相仪式系列</t>
+        </is>
+      </c>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="L42" s="12" t="inlineStr">
+        <is>
+          <t>P3-E-3-The-Hoodwitch深度拆解.md</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>参考：现代巫术美学品牌调性 × Bri Luna创始人 × Witch Tips每周运势 × 月相仪式系列 × Squarespace</t>
         </is>
       </c>
     </row>

</xml_diff>